<commit_message>
arg_test removed because not very used finally.
</commit_message>
<xml_diff>
--- a/dev/TODO_backbone_all_args.xlsx
+++ b/dev/TODO_backbone_all_args.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gmillot\Documents\Git_projects\safer-r\saferDev\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87CCE893-76B9-4F1C-869D-917DC313CE89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21A4E32-0A48-454D-BE3F-DFAC9BAAFD79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{07E7905C-C0FC-435A-9AE4-BD70C30EB32A}"/>
+    <workbookView xWindow="19720" yWindow="-15670" windowWidth="28800" windowHeight="15450" xr2:uid="{07E7905C-C0FC-435A-9AE4-BD70C30EB32A}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -856,74 +856,75 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:27" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="P4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="U4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="V4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="W4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z4" s="2" t="s">
+      <c r="B4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="T4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="U4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="V4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="W4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z4" s="4" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
backbone v19.0 rechecked -> ok
</commit_message>
<xml_diff>
--- a/dev/TODO_backbone_all_args.xlsx
+++ b/dev/TODO_backbone_all_args.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gmillot\Documents\Git_projects\safer-r\saferDev\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21A4E32-0A48-454D-BE3F-DFAC9BAAFD79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C81699C4-3D4B-43B6-B8C3-D90BD614C744}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19720" yWindow="-15670" windowWidth="28800" windowHeight="15450" xr2:uid="{07E7905C-C0FC-435A-9AE4-BD70C30EB32A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{07E7905C-C0FC-435A-9AE4-BD70C30EB32A}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="51">
   <si>
     <t>all_args_here.R</t>
   </si>
@@ -213,6 +213,12 @@
     <t>help pages
 other functions
 \link{try}</t>
+  </si>
+  <si>
+    <t>backbone v19</t>
+  </si>
+  <si>
+    <t>vignettes</t>
   </si>
 </sst>
 </file>
@@ -615,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39A2B6C9-DACA-4606-B471-C75D7DA26424}">
-  <dimension ref="A1:AA22"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.28515625" style="1" customWidth="1"/>
@@ -631,7 +637,7 @@
     <col min="22" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="153" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" ht="153" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>34</v>
       </c>
@@ -710,8 +716,14 @@
       <c r="AA1" s="1" t="s">
         <v>48</v>
       </c>
+      <c r="AB1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="2" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -778,11 +790,23 @@
       <c r="W2" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z2" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="3" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -852,11 +876,23 @@
       <c r="W3" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z3" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB3" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="4" spans="1:27" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -924,11 +960,15 @@
       <c r="W4" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4"/>
       <c r="Z4" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="AA4" s="4"/>
+      <c r="AB4" s="4"/>
     </row>
-    <row r="5" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -977,6 +1017,9 @@
       <c r="P5" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="Q5" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="R5" s="2" t="s">
         <v>22</v>
       </c>
@@ -995,11 +1038,23 @@
       <c r="W5" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z5" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB5" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="6" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -1069,11 +1124,23 @@
       <c r="W6" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z6" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB6" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="7" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
@@ -1122,6 +1189,9 @@
       <c r="P7" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="Q7" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="R7" s="2" t="s">
         <v>22</v>
       </c>
@@ -1140,11 +1210,23 @@
       <c r="W7" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z7" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB7" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="8" spans="1:27" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1214,11 +1296,23 @@
       <c r="W8" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z8" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB8" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="9" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -1288,11 +1382,23 @@
       <c r="W9" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z9" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB9" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="10" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1362,11 +1468,23 @@
       <c r="W10" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y10" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z10" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB10" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="11" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1436,11 +1554,23 @@
       <c r="W11" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y11" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z11" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB11" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="12" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1510,11 +1640,23 @@
       <c r="W12" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y12" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z12" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB12" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="13" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1584,11 +1726,23 @@
       <c r="W13" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y13" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z13" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB13" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="14" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -1658,11 +1812,23 @@
       <c r="W14" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y14" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z14" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB14" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="15" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -1732,11 +1898,23 @@
       <c r="W15" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y15" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z15" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB15" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="16" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -1806,11 +1984,23 @@
       <c r="W16" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y16" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z16" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB16" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="17" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -1880,11 +2070,23 @@
       <c r="W17" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y17" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z17" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB17" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="18" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -1954,11 +2156,23 @@
       <c r="W18" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y18" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z18" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB18" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="19" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
@@ -2028,11 +2242,23 @@
       <c r="W19" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y19" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z19" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB19" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="20" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -2102,11 +2328,23 @@
       <c r="W20" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y20" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z20" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="AA20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB20" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="21" spans="1:26" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>19</v>
       </c>
@@ -2174,9 +2412,13 @@
       <c r="W21" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="X21" s="4"/>
+      <c r="Y21" s="4"/>
       <c r="Z21" s="4"/>
+      <c r="AA21" s="4"/>
+      <c r="AB21" s="4"/>
     </row>
-    <row r="22" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>20</v>
       </c>
@@ -2225,6 +2467,9 @@
       <c r="P22" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="Q22" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="R22" s="2" t="s">
         <v>22</v>
       </c>
@@ -2243,7 +2488,19 @@
       <c r="W22" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y22" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="Z22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AA22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB22" s="2" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>